<commit_message>
Adiciona as duplas originais
</commit_message>
<xml_diff>
--- a/duplas.xlsx
+++ b/duplas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{520FB2D8-3206-4105-8077-3A9CD7DCFCA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9343FBB-6FE3-43DA-9770-FBE9489ECBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>duo_id</t>
   </si>
@@ -57,6 +57,114 @@
   </si>
   <si>
     <t>Vinas#OVN</t>
+  </si>
+  <si>
+    <t>Kennzy + Guiven</t>
+  </si>
+  <si>
+    <t>Esa + Brucer</t>
+  </si>
+  <si>
+    <t>FNB + Minerva</t>
+  </si>
+  <si>
+    <t>Squallzera + Ammy</t>
+  </si>
+  <si>
+    <t>Luma + Onika</t>
+  </si>
+  <si>
+    <t>Ayel + Revolta</t>
+  </si>
+  <si>
+    <t>Gui Atlanta + Peu</t>
+  </si>
+  <si>
+    <t>Arthur Lanches + Imaaaster</t>
+  </si>
+  <si>
+    <t>Imaaaster + Yap</t>
+  </si>
+  <si>
+    <t>Kennzy_Guiven</t>
+  </si>
+  <si>
+    <t>Esa_Brucer</t>
+  </si>
+  <si>
+    <t>FNB_Minerva</t>
+  </si>
+  <si>
+    <t>Squallzera_Ammy</t>
+  </si>
+  <si>
+    <t>Luma_Onika</t>
+  </si>
+  <si>
+    <t>Ayel_Revolta</t>
+  </si>
+  <si>
+    <t>Imaaaster_Yap</t>
+  </si>
+  <si>
+    <t>Gui-Atlanta_Peu</t>
+  </si>
+  <si>
+    <t>Arthur-Lanches_Imaaaster</t>
+  </si>
+  <si>
+    <t>guiven#vasco</t>
+  </si>
+  <si>
+    <t>hamburguesa#esinh</t>
+  </si>
+  <si>
+    <t>Brucer #oreia</t>
+  </si>
+  <si>
+    <t>Azul#999</t>
+  </si>
+  <si>
+    <t>Minerva#IDL</t>
+  </si>
+  <si>
+    <t>Squallzera#BR1</t>
+  </si>
+  <si>
+    <t>Gostóxica#ammy</t>
+  </si>
+  <si>
+    <t>cobra solida#luma</t>
+  </si>
+  <si>
+    <t>SupremaOnika#COVEN</t>
+  </si>
+  <si>
+    <t>AYELGODLIKEMODE#PIT</t>
+  </si>
+  <si>
+    <t>chico lanches #rev</t>
+  </si>
+  <si>
+    <t>Atlanta#BR1</t>
+  </si>
+  <si>
+    <t>RED Peu#Auau</t>
+  </si>
+  <si>
+    <t>Arthur Lanches #13777</t>
+  </si>
+  <si>
+    <t>iMaaasTeR#br1</t>
+  </si>
+  <si>
+    <t>PIJACK#GOD</t>
+  </si>
+  <si>
+    <t>Yap#123</t>
+  </si>
+  <si>
+    <t>kennzy#knnzy</t>
   </si>
 </sst>
 </file>
@@ -428,15 +536,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705F9F5F-280A-4165-8E5D-B53A8F474D62}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -450,7 +559,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -464,7 +573,134 @@
         <v>5</v>
       </c>
     </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix nome da dupla do pijack
</commit_message>
<xml_diff>
--- a/duplas.xlsx
+++ b/duplas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9343FBB-6FE3-43DA-9770-FBE9489ECBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D304E863-A907-4633-9A8E-2AE104366C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
   </bookViews>
@@ -104,9 +104,6 @@
     <t>Ayel_Revolta</t>
   </si>
   <si>
-    <t>Imaaaster_Yap</t>
-  </si>
-  <si>
     <t>Gui-Atlanta_Peu</t>
   </si>
   <si>
@@ -165,6 +162,9 @@
   </si>
   <si>
     <t>kennzy#knnzy</t>
+  </si>
+  <si>
+    <t>Pijack_Yap</t>
   </si>
 </sst>
 </file>
@@ -578,10 +578,10 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -592,10 +592,10 @@
         <v>17</v>
       </c>
       <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
         <v>26</v>
-      </c>
-      <c r="C4" t="s">
-        <v>27</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
@@ -606,10 +606,10 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
         <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>29</v>
       </c>
       <c r="D5" t="s">
         <v>9</v>
@@ -620,10 +620,10 @@
         <v>19</v>
       </c>
       <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
         <v>30</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
@@ -634,10 +634,10 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
         <v>32</v>
-      </c>
-      <c r="C7" t="s">
-        <v>33</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -648,10 +648,10 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
         <v>34</v>
-      </c>
-      <c r="C8" t="s">
-        <v>35</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
@@ -659,13 +659,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
         <v>36</v>
-      </c>
-      <c r="C9" t="s">
-        <v>37</v>
       </c>
       <c r="D9" t="s">
         <v>13</v>
@@ -673,13 +673,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
         <v>38</v>
-      </c>
-      <c r="C10" t="s">
-        <v>39</v>
       </c>
       <c r="D10" t="s">
         <v>14</v>
@@ -687,13 +687,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
         <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
       </c>
       <c r="D11" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
add zero e art test
</commit_message>
<xml_diff>
--- a/duplas.xlsx
+++ b/duplas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D304E863-A907-4633-9A8E-2AE104366C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2849DE21-2EBD-4BA6-AD67-865737F542D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>duo_id</t>
   </si>
@@ -165,6 +165,15 @@
   </si>
   <si>
     <t>Pijack_Yap</t>
+  </si>
+  <si>
+    <t>ZeroArt</t>
+  </si>
+  <si>
+    <t>Arthie#BR1</t>
+  </si>
+  <si>
+    <t>Bagtan Zero#br1</t>
   </si>
 </sst>
 </file>
@@ -536,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705F9F5F-280A-4165-8E5D-B53A8F474D62}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -699,6 +708,20 @@
         <v>15</v>
       </c>
     </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix nome do zero
</commit_message>
<xml_diff>
--- a/duplas.xlsx
+++ b/duplas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2849DE21-2EBD-4BA6-AD67-865737F542D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0CAA76A-843D-4C51-A981-61B001173A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
   </bookViews>
@@ -173,7 +173,7 @@
     <t>Arthie#BR1</t>
   </si>
   <si>
-    <t>Bagtan Zero#br1</t>
+    <t>Bangtan Zero#br1</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
fix nome dupla pijack
</commit_message>
<xml_diff>
--- a/duplas.xlsx
+++ b/duplas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0647A7-FC22-42E8-8AC5-072F0425F8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EE3868-F690-42EC-9EEF-720BA07373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
   </bookViews>
@@ -74,9 +74,6 @@
     <t>Arthur Lanches + Imaaaster</t>
   </si>
   <si>
-    <t>Imaaaster + Yap</t>
-  </si>
-  <si>
     <t>Kennzy_Guiven</t>
   </si>
   <si>
@@ -156,6 +153,9 @@
   </si>
   <si>
     <t>Pijack_Yap</t>
+  </si>
+  <si>
+    <t>Pijack + Yap</t>
   </si>
 </sst>
 </file>
@@ -552,13 +552,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
         <v>4</v>
@@ -566,13 +566,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
         <v>22</v>
-      </c>
-      <c r="C3" t="s">
-        <v>23</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -580,13 +580,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -594,13 +594,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
         <v>26</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -608,13 +608,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
         <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -622,13 +622,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
         <v>30</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -636,13 +636,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
         <v>32</v>
-      </c>
-      <c r="C8" t="s">
-        <v>33</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -650,13 +650,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
         <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -664,16 +664,16 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
         <v>39</v>
-      </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
commit certo e parango dupla
</commit_message>
<xml_diff>
--- a/duplas.xlsx
+++ b/duplas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EE3868-F690-42EC-9EEF-720BA07373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269CCA5B-A5FF-4162-8ADE-115B63EF0EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>duo_id</t>
   </si>
@@ -156,6 +156,15 @@
   </si>
   <si>
     <t>Pijack + Yap</t>
+  </si>
+  <si>
+    <t>kmyzth#mafer</t>
+  </si>
+  <si>
+    <t>Vinas#OVN</t>
+  </si>
+  <si>
+    <t>ParangoDuo</t>
   </si>
 </sst>
 </file>
@@ -527,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705F9F5F-280A-4165-8E5D-B53A8F474D62}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -676,6 +685,20 @@
         <v>39</v>
       </c>
     </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fim do teste parangoduo
</commit_message>
<xml_diff>
--- a/duplas.xlsx
+++ b/duplas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{269CCA5B-A5FF-4162-8ADE-115B63EF0EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D164CCB-7D99-4892-AC41-447CE54275FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>duo_id</t>
   </si>
@@ -156,15 +156,6 @@
   </si>
   <si>
     <t>Pijack + Yap</t>
-  </si>
-  <si>
-    <t>kmyzth#mafer</t>
-  </si>
-  <si>
-    <t>Vinas#OVN</t>
-  </si>
-  <si>
-    <t>ParangoDuo</t>
   </si>
 </sst>
 </file>
@@ -536,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705F9F5F-280A-4165-8E5D-B53A8F474D62}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -685,20 +676,6 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" t="s">
-        <v>42</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
atualizaçao dupla kennzy sulas
</commit_message>
<xml_diff>
--- a/duplas.xlsx
+++ b/duplas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Pictures\Arena Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D164CCB-7D99-4892-AC41-447CE54275FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4F7EA1-6F0B-46B3-9A6B-CAC9418BDB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4EECEE7B-0D3A-4C28-BE97-B907C1A3E606}"/>
   </bookViews>
@@ -50,9 +50,6 @@
     <t>duo_name</t>
   </si>
   <si>
-    <t>Kennzy + Guiven</t>
-  </si>
-  <si>
     <t>Esa + Brucer</t>
   </si>
   <si>
@@ -74,9 +71,6 @@
     <t>Arthur Lanches + Imaaaster</t>
   </si>
   <si>
-    <t>Kennzy_Guiven</t>
-  </si>
-  <si>
     <t>Esa_Brucer</t>
   </si>
   <si>
@@ -98,9 +92,6 @@
     <t>Arthur-Lanches_Imaaaster</t>
   </si>
   <si>
-    <t>guiven#vasco</t>
-  </si>
-  <si>
     <t>hamburguesa#esinh</t>
   </si>
   <si>
@@ -156,6 +147,15 @@
   </si>
   <si>
     <t>Pijack + Yap</t>
+  </si>
+  <si>
+    <t>Kennzy_Sonlas</t>
+  </si>
+  <si>
+    <t>Kennzy + Sonlas</t>
+  </si>
+  <si>
+    <t>Rock Lee#jesus</t>
   </si>
 </sst>
 </file>
@@ -552,128 +552,128 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
         <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>